<commit_message>
cambio de imagenes a webp
</commit_message>
<xml_diff>
--- a/tenis.xlsx
+++ b/tenis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\PROGRAMADOR FULLSTACK\PROYECTOS DE PROGRAMACIÓN\PROYECTOS PARA MI USO\tienda_triplea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{345E5B46-1DD8-4600-A907-22433E93DBE1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40743F63-9EC3-49C8-AAC9-57CDDA0B8BC6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="1" xr2:uid="{B81BA034-5AA5-4E31-BF73-0823AFB888DA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="2" xr2:uid="{B81BA034-5AA5-4E31-BF73-0823AFB888DA}"/>
   </bookViews>
   <sheets>
     <sheet name="DATOS DE LA PAGINA" sheetId="10" r:id="rId1"/>

</xml_diff>